<commit_message>
chore(gt): QA approves the 39 test cases and the catalog
Import QA's Excel review (all 39 test cases approved), set the catalog status to
approved and re-export the xlsx so it matches test-cases.yaml.

Still open: module-map.yaml is draft (route paths to fill), AC-1.7 and AC-8.3
have no test case, and the technique/api coverage thresholds are not met, so
qc-agent gt validate still exits 1.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.qc-agent/ground-truth/test-cases.xlsx
+++ b/.qc-agent/ground-truth/test-cases.xlsx
@@ -684,7 +684,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>b4e5c1f22558a2e7fc4bdc834cf286aea1e54f6e28ab5e6f7cbe1f7e0d5444d9</t>
+          <t>e06f1d34178ed9cec7d4cbce16894f75b8157803617b0e2be778fe92688d4562</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>eNrtXeuPG1WW/1dK1koQjR2Xy+VXVvshk2RJdgPJJA0LM0Kt66pr16XLVaYeTpso0iA+oNUIMRE7GiGEhtCKosBEwGQQmm6N+OBs/o+ev2TPOfdW+Za7bHeHJrNSjMD4Uafuefzued1bt29XnDAY+MJJ4sq523eqlXHkwpuKgNfKhHksqFQrscesVhu+aA9si3G3z1tN0+70BoOm3ej32KDvNHnftru9jtW3+4Mec1p9p2HZcKnb6NoWHzgDp+t2KzBAnLAkhcEqbsQGCdw94XGy7bCYIweVrQu18xdqjbONWmvQbVsD/I452xEfwM+/qcjfKm9XK3wiXB44HL6FTzsiQI7ZWGwP0sBJRBgwH24ehAneN0h9v1oJIzEUAVzm+6MKispBeFfgxfk140jAZck0+xwxeS+ef8Hf4U7CXWCJxWGQfX1ErDjhY2T5doXvjoECBXmHCOCrcAxXBhyZYIkH7/8F3k6Yn6ph7rw9v+NvbLNRtS3r7Ts4+LspqGt+r9twgzi+FaLVKreiMBji54bVhPulMY8CNuI4VBjwXQEsBck2fr29O30PjTHiiRci6fVrN7fm3NRBj3WWJl7dD1Fjd5CfhDteIN5Nc00kIkG1VJ78/skHwdAIvMP9R2NjcnjwmTCysesZe0bMhNE/PPidkRwefG043uHBXYEsZAa3anar0Wg2ygxuAWv0pvcCWt5sLrN8FA6Ez6+40sC1zMI19UMFqcacAVElRH3BnR2Pu6nP3fP4pWX2ejWzAf9umeY5+vcXZgdecVaKEX8PUAOXnY8Fq18Oty94YvtVEXjrgBOlQS0bKF6DnVcODz4SxvnrVwAW+/dCwweEOJ4xmn1h7HizvwKsnNljY+yJ2VeBAZjZG+MlH0qwBcux5LTaTtPcYOm4WHL5QAQkwxs8igV+2QC5pfeIvTD13dqACX+d7QF3CY8yBJ7U+pLaUNTGy2jZh44RkH9h7kgEZwAWAiz+9FtmPLmr+51VvqVZG3CbOXYZHpovFgws01yAwNoYwEADE5TiuMbMCIxx6PsCTKSm8nD25RSn7x8FGO3pt/MfnFAYPkx5LwQYJGDYw4NP0bLDp98eHnwuDHf2N/iYeDw0rt+4qFvWrnXMLm+0yixrL7XswA9vvbj2hJgepglYs/pzeZWchVculXIAXmU1lm6ylCa6muK76eH+/aRqJOEOD7JoICe8l2JY+ERkUErg0wfGMMfik7uIoT0HLt/fCzE7+VDHT6vWarpdq1eGn9YmzZwHCCeNIsgtrs+zzdB3s+RO5psBv6X9DEEjSo6VY+YZ7Lo08/DgD8IYgbdPwNqH+w9T+IDJZjA83P8G0oOn9wKjYRk7s79jIPhuZUho1dpmt9+wN4Y/seFjyApWWn7h9+eCgSSiGFH4xRMw2wPKLVbXHu1ap8lYt7TYbL+QaeLxCk64iVhwAlFIhhrxUZ9HxSJ0HRDw0nUZ4xblicnsC3T4kC3sBQsFpxFBfgFAWGXubs3u2y2zNGnobsxdNPdpFYJ1vFGN7nTcPBLzQJjtGQdZcYiJwcricLntrbNQ7YLp2/2jtrdeyL7SSXK3kxV3VyFnmxouCzwjnt0Duy1Udycv5NB6/XbLNHsb6x1j5s5retnaLanxe/BPXua/PnZZAg4UdIi/GtiYLU7x19cgon5bvdsW7h116faYRWwUaw2rbbGsY1UTmACsRJVicgFLMgbknK/uNSKMXMtqNvgGRqcDo3mr6HT7Q1tlXSFp6wR9fhJh4j9cY2ve6vSZu7H1adua/ZP/eb5Ym1AfITHeTWf3oMo0j1NmAsLMGjebbbNZCj9zg7+FpOPipauXti49hyhTrcDg0RQJsrBB4XBN+Hlz9pj9xOBj1RrWAOrNMkRYG0CscEgVB7gNXBa9xVlUOWeZll2tSGNIfgaC+6ismzAAsjAKXTTaQOxyN2ODlD1p4EdcCppg0Tqx8aWFL2186eBLF196+NIw6ZVoGkTUIKoGkTWIrkGEDaJsEGmDaC2iteR4REtl8sQiWotoLaK1iNYiWotom0TbJNqmZJZom0TbJNom0TaJtkm0TaK1idYmWptobSkp0dpEaxOtTbQ20dpE2yLaFtG2iLZFtC2pJqJtEW2LaFtE2yLaNtG2ibZNtG2ibRNtW+qYaNtE2ybaNtF2iLZDtB2i7RBth2g7RNuRBiLaDtF2iLZLtF2i7RJtl2i7RNsl2i7RdqV1ibZLtD2i7RFtj2h7RNsj2h7R9oi2R7Q9CQ2FDQkOE3IJxPbuefA2gLlXwyDx/kvECMNp9h3b4VFlXVi9tOtw7hoSrIYvRiJ5bpFODVqIdUNBP0Fxhu1V01zj3Not3u5unNtPdW6oghqrBanqo/10XF0JqF1nTOH+mdmfG7CCJx+MKDLuAJo+SA338OAbwPbhwYfpGjz1HbPtOBs8nRhPabAThLeCf1cxUd72uCDBtt2IPXeYYMfvd4FnBEPvyUMG/wux06uYWYUTuzbgUOeVptn2BidFnCymSZA7Q3r8hsqObt85mbXr4Viq5DjtQHltZnxsASaeONz/MTWIKdoB8IMDXzJwF2BkXLb9JjH66eHBp85KBHRqzWbbKdswCL9tEHAaafXrQZyOx2EEwpBXefOtX69KstlpZUTauAomUfocnZIcUq04AO7+iH2ng701aLS5OWjxDRpPBY1OOOqLgGS5QbsKy6o9UDJgZyvUvkqmYzQujikiQMypwPEm9wdQ7g+eLwo1FdDAsvdEjtJRLnQ5IJtnG7Wu6TJekkg1N23QVTtr43DET7Cj1jL/yTtqt/R9tKp/6dEuuqFggSzpdnBf5Rq49JomL9ses4HLacLlyAbsnw0KWZ6Vr6avMr9VazWanbIdEs1N2fVzmv8XZutcc8FbXEqjcMzrV0FbMODP7CoydJwk3UG8dK2uaQ82eDklvLhM+NP/jw9slGBGMp13dpDzlWDp1ey2yVmvDCy9FxQspg3/9U68MlbcYXU7e1u+MKb9urgylv10jA0YtAKW78SSe64PDz7JtlmqAl79gv2cB/AK0Hg/JYR8GKzAhg15h9UY8EFJmmpv8o7j7PAHRAQ8qsO1Ka87PhOjNRP6Al5j4POXSzbWyTseb3+dfbZZ63Y7vKwRZ79oj9qsjwQgRhIxJ8mLTLkw+U7YP/pQH3y5dgOtqHmc+bidGvTui6GXrDH+9ew65cphkLJJvcrgrZprsVbbLjN4a2PwBYOzceJ47Ip6fqIG732fB0NyvM9ueDXpQyeqAzPROqv/knqq4Jv3H6TGtQs3sg5Dxlw9Z8tw/vdh5tJPjI0W7bNrO2ZJF6y18ebH8eZ9BhapSWce8xidBIZ5+Q6jfH3M0piXxPr8kiOhXv5yjEh/HW9tqOtPanqrZrX7zZ5VZvpNRXAqpo94nI5+JtvfoHs/m/Hb2D3q9xtmifHbm3l/nIckgyBlfg0KqzBK4oq2V81lCWRqWAtOuCccrNeqlWneKV+Xu/OR0Z9B/ebgy3wD/kkfo2iftWtmz2kzs8zCm/XWU7fwmA05LUHgm5viPfwAwx7f8m/NvkoNhwL+2Jt9iVunGUzo4qZW0zTc2V+CYV3+uGj/LBHQNwTpmGjXeo225TbKMNF+gev6Z8dFHfjAp2jXwSOm5a5zlZvhiGdLX8eGxiUaQy06cVc+Zk93BMAc3FdPVONW+z1MFN8v7N3BlYTPxgsVvg6KTq3ZMLtWuwwUL+pC6OpGz2mB4qQAgJQ/XyTAQ6FENDrv+/+WROmRzgBhrH5j6xokCCzCxYU5OuT5Druze446pEVHQw8Kgka7XYqG3sZFnA4a5sarnBswP+bV1V7jtTC4pDJEMuybb/1aPsv7zC5EgwoFlMxNaDABsefA6EDG2LG6TVay4NTZPJZ5MkBgT9gDc4bRuhNbbqSBcVleSSH+v+UZO8YuH1UN+QR3FvNP9qBmB8/V6DhN3iyzZ2tz4s5SW85beIp+zdOQV4zLdDlNrXt0/snsntAnWqJKN7CrK9gwCONEOLFuq07N7Fidvl1mq85m7q05zsYV69ptdCQSXleYZBBXp5iRPxpXn/Vp9i4edNbstFjnqOm6L1qX5UTTDLhy13nHS4E7DkWQGHixCHgcF6ZVYb7Fh/vfB0Y8+yIY4rlKFVBuOMFQiHzIZ/2gLKq8MXuE2fN93N+MmfKIzi+azmszPbXGvPs7B7stP0rzv3H+8vnXoFRj2ZLMy5iBUbqOvwMzFL7P6KfnqeSdtorRyi2SX97aum44mO/RSVsO4IxgOPZkvi83205mX4QFhoJhSv0fuSv7rDxHzzrbRMHwCkffLUDd5alaAHQwG/RD6hvJ3ZRaZYGSB3L1eIRlKbHoQMLihxBqgBXqNX2K/BxDP/8KQ9IxY3D1CMgSeXli7My+kocRwLf3HRz1fmp4sz8Hnj79PDChZ0yE1FGEcxEKYXkH/F2yzOKYQ76jCYHMwcCPac1TnjiVK6hVrL81ScF9R0Dok2Jgsn/HaI5/FGACrg7AoiMwHI/JA9Iy9oaCgXHkeioU9I+A0BeQwFWLhgdVIizvJaRUdEQ8Q7Vu+pxVPOT1cjYG7eitC0jpsBbUUOrJlf5giNZw8BAWr8Teaqv3ehjjPu9gWF2ELB30AlNZrk3q7GZXFvF6DKh251BFfvdG6lSwlwKYxSCEhCLOycTTByIXDC8fG7MvR/Tbg9FLGsQyFpLZI3x4YY5ZoH8sayFw+R4JLbGDmvmPm9dey0CjTdk+lmCJAmgSzfYd8EDxGLyvXpDnMvXmMkmd4ZiIo/Rw/yEEEvxQqq+ENgGSayhAby6Wg9vzFTf4HAbq7IdEl+9lj8WeCIb1IIxGzBfvURw4o88oh87+mAMR3QPiAe87nrujowqIZt+XKkFJ3tQdjzanBsBJdicNs7fCaAew5oQpYH8iBwPNyK8v0Lc+HzJnmtFKWHs4l/+EugtDvzgF8WhcZ8HYy2ae1GduRpIY/MS9AAF9sMb68yFy0e2iS8m2b0TG7uHBI2Dz79kODXf2NyNhfYTZ3txBzf6C7buDjwXZ/PPCBlE1X9HWP0ofpG6lvpHPAaIG5yLmOgFW3w8WZnJum5DO50JFkLrmUSihUz4lE7mIC15TMXENchmoSWA8RPv9RFuZQBjv/zBW3vSokEclUqLGSOugXFNjN0RPpM1sQURgCAwUMtYeVVbx7EGBSYJ0VDm8gyGbqu9I2lxM9Lj/OUev47PRGK6efTE1rF69adabDdWoT6dwVUAJByoSt6/704KcJQaZI2MZ78hi4Mn2nbz3EvtpRsrlysXo4BM+5HOHc1bpoT/plNQWt7rSvPxFugBibK7xdyEtVupWWRKdKX2fvNdD6eTGR6Vx0UERNqt4RiguXOOJo6A58iP5MscAcjyIEhNuZKlxde4eYbLIxBujTVmYPyI3RpSLImZ9n8OtkzTiGNVimh99OotOwjHgu4lBa/NUPd+XLfegYD6SyZ19LxaSS6UzHHtR4mOYCrj4Di7Qcz70O4TSQMlh41EUuTNFpanzlWUzT24PAO6HvO6ELq+7PGHC1xWD9tPCBfjGIR78qnnHkuRSxf8sQwDyfhTeAp0v8yDrIgc1nLQ0QLKvZyC7IPXUiFguuIX1gf6E84hoFGu5O01oAeTJ3cyVU07i0JGDPvpo3Y6j2V9J2o+pVSJnVlFUhNcnSrzPM/0q2WXqAYlcYW0GTzTcUwchK3Xohu37zNmp9cPdcuvaet6DDOVP4BHmjpiGGPzIUdi9eO1VNSHmmUwhEh41INS7STiSD6toGADAPMjSvtzGc6+Vn9W6mKzmgrS1kC+psUjAXAeNhltZsN2xNDOjyk0mJAjyYoGxDHSyICnGbsScShbzMp5u52HFjjeAjDbnulMMZZhz9MNwx5Ct22LqjNpPx37IcCGGFOyonZSao5g9Agmkp5pkp1+iw3TR8X6Y6AaR2XaGqaWBSoZU6k+oPLW8SMxlQsd3nVYSVXX02rXti+e3zuudC8mbmoRixMM0qW9dvVm3TXvphJFXjzL/p9UOlD/QZMii8Vz1JOXClBnjfB4hPpUpVdbFqbvy6bh8qvSK8XiH3Nm7KWoKyp1HQs6JukomRoiugPSlBsGYkohkWi/68GXiRgzymby/UhAYl1m/YQsepCpLChlUCzVRbjNdrGWOkdyXHExJ3qJ0+gZPoqkcWV6TiUO49Kk1JVXCkoSPxpjOo84/K3pAyvuBvI57xnSZKA1VqRbeMZGxsE9+Rr/VY2VvfT5VlzY1yhWhBYZ1wSdXgl00fwZqvQ5EL8XkPSa0uBGR0iRwy7QgpdaT1mzS6gjJhjqK+aIOSkTRpvtcKpjvuVSYS7+ZhTJ1iStiwF3AnUQGgSFCse5zxXApWkcy5SYABBQRixNVZtIFJ3+SKKZ6dwrBKCJ42FwIypTBDkKqAEZjKbplSqrk3xA4+Nq4+aurBfazC3QOIUBNQAPFGqZojXVhoeghZaeGUe5L2O6rcoHOr88jQYsiQd5fQSqpUaVF6atP7hnVIdh6y6O0m1JkOlFJzxxchksTMHeY+PWjnPcunb+c9dZwyr2vDmY3Xn7y+zfPqCQ7iQQl/zseE/mR/dXSHlth7KKbmKtajd+WKao2N6WJ3JS0nmee9MQsHqHjGy8nAoMucVo14nQ0YtG0mp8x4UpN0ikDoNvPgjMF1Y9ZFHN5O0iGYd7TvpkVgC5v7MjZQNkPNbNkNQjl3Vwu7AxfffptXuPGOFNlXKM0XPYroJBzdkAIpRx8vSvyR38h2ca7qwoYL396j8D4YxmU0QrUzCF975X3mrBuirCjXayGytzrk7vhjGIOBWeQYi6cdZy2t9VSO4+WNnjJherbD4+6Rjn/syCyPFgU+oRYZy9MC61PUd5+zIWztM63UMU5IuWlf/z2f14C7YcL4khTTRaaPYHx2utXr2bZnllMrQv3ff3Kql6v5plyGxISKSVe319bbMznYjZ1p3XBx+ODdrF3tvBYTzL78wjf7/84IhmSp98+JVeFRcMy1hGJeUu6pOde6gkwnF3WFZMhAHv8VxnYLKVTYt06PeQfG7dEAvOdJWwheq7psa5cciBEymm3dF7NpxB2JVmiFpB8qvr0WZWLhk72MmWn2g4alS/A4A/Af12KHTbmVbilk8bLVwWO/PEUiqZgiDUBDSKp4qZDAC8oGoTeVw5BO6aH2v3Sjyo9HR78AdWBKeA4Ch0OQrr13Ar1IJT/x78oxN0jSRPkDkdVrfInJSspRDcNXaOQvdQHLM0Vc4mbC+m/1sf2ssj0KQbhrxcW68hr6Bsq0DAT6RzmZXMWpKGUuLuwYqE11S/+UiVwuq/AcmYP4n/o7JxZucpT1mUu5lIdSnMvQbLpUuMfJgAeputFYTr0xlCk0R/w4Qb32ThesM98LLW6psKhSnx0sy00rKrZYyaoDWmiz6ULh3qRHmPAPQ++f7KeVi5Se7EglV1f9WhMn+bR2GdBgH0pvTK9xfuxSHhBF2oA+vtTyIlyZfLTsgQtoaQPXcvdPF3T9aE3MFUdp2KqyhVKVgrIgR/xyd2zmDNcJpRT0Nz/Oigs0ci/iaH6dtyBCiWuAgKHcp0+K72y5R/cnfUnkf/ZJXLeeDMFzQnpjiZedQGNuefB/Hu+PrrgU3KubflkAcwPLisXcA7vUAVCPRllOJntZO3uiA0GwiGmtNawxhP17VCrDxRmHsiWyYoYo0cV4nLeP8OQL/KMvUux5pXZY8Acuh9ysMopKz8rRtgWzU9/VY1fHT0uH/vhdIUE9QtXahcuPptus6KpPl8eu1Ot3GIwfyN5mNf/AfnNrx0=</t>
+          <t>eNrtXVuP20aW/iuEsEBijGRRFHXzYh88tjf2rhN77U42mUHQKJElsdIUqfDSbsUwsEEegsUgyBjZwSAIgonTMAwnYyQZTxBMNwZ5kNf/o+eX7DmnilRRoqRuT9uzgBUkii48rHP56tyqWH274oTBwBdOElfO3b5TrYwjF95UBLxWdpnHgkq1EnvMarXhi/bAthh3+7zVNO1ObzBo2o1+jw36TpP3bbvb61h9uz/oMafVdxqWDZe6ja5t8YEzcLputwIDxAlLUhiswsbjKNzlLgyQ8DjZdljMkYnK1oXa+Qu1xtlGrTXotq0Bfsec7YgP4OdfV+RvlXerFb4rXB44HL6FTzsicOm2YnuQBk4iwoD5cPMgTPC+Qer71UoYiaEI4DLfH1VQWg7yuwIvzq8ZRwIuSybZ54jJe/H8C/4edxLuAkssDoPs6zLJ4oSPkevbFb43BiKU5T2iga/CMVwccOSDJR68/yd4u8v8VI10593ZTX9tm42qbVnv3sHx309BY7N73YYbxPGtEG1XuRWFwRA/N6wm3C+NeRSwEcehwoDvCWApSLbx6+29yQdokhFPvBBJr1+7uTXjpg6qrLM08ep+iEq7g/wk3PEC8X6aKyMRCWqm8uS3Tz4KhkbgHR08Ghu7R4dfCCMbu56xZ8RMGP2jw98YydHht4bjHR3eFchCZnOrZrcajWajzOYWsEZvei+n8c3mMuNH4UD4/IorbVzLjFxTP1SQaswZEFVCVBnc2fG4m/rcPY9fWmavVzMb8O+WaZ6jf39hduAV56YY8Q8AOHDZ+Viw+uVw+4Intl8XgbcOO1Ea1LKB4jXwee3o8BNhnL9+BZBxcC80fACJ4xmj6VfGjjf9MyDLmT42xp6YfhMYAJv9MV7yscRbsBxOTqvtNM0NnE4AJ5cPREBivMWjWOCXDRBd+pDYC1PfrQ2Y8NeZH6CX8CgD4UkBIKkNRW28isZ96BgBeRnmjkRwBpAhwOhPv2fGk7u691nlYZq1AbeZY5dBovnSIcEyzTkUrA0GDJSwi4Ic154ZgTEOfV+AldSEHk6/nuAk/r0Auz39fvaDEwrDh4nvhYCEBGx7dPg5Gnf49Pujwy+F4U7/Ah8Tj4fG9RsXdePatY7Z5Y1WmXHtpcYd+OGtl9qkEN/DNAGDVp+Xb8lZeO1SKQfgW1bD6SZLabqrib6XHh3cT6pGEu7wIAsLctp7KcaHz0SGpgQ+fWQMczg+uYsw2nfg8oP9EDOVj3UItWqtptu1emUQam2yzkKkcNIogjzj+iz5DH03y/Vk+hnwW9rPED2i5FgpZ57Qrss6jw5/J4wRuP0EDH508DCFD5h7BsOjg+8gVXh6LzAalrEz/StGhB9WxoZWrW12+w17Y/tnsX0MGcJK48/9/kJgkEQULAq/eALmfEB5xupqpF3rNBnrllag7Zc1azxeFQo3EXOuIArJViM+6vOoWJmuwwJeui6B3KK0MZl+hZ4fMof9YK4KNSLINQALqyzerdl9u2WWJhDdjcUXLH5a1WEdb1SjOx03rcS0EOZ8xkFWMWKSsLJiXG5+6yyUwGD9dn/R/NbL2nI6SSp3sorvKqRwE8NlgWfE03tgurmS7+TVHRqw326ZZm9jwOPN31mtL9u/JbV/D/7Jy/83xy5LwJOCGvFXAzu3xYn+5hpQ1G+rd9vCvaMu3R6ziI1irZe1LZY1s2oCk4GVwFJMzsFJBoOc89WdSESSa1nNBt8g6dSQNOsinW7raKusYSTNnaDzTyIsBYZrzM1bnT5zN+Z+DuZm/+B/Xizcdqm/kBjvp9N7UHqax6k9AWRmjZvNttksRaC5geBiAnLx0tVLW5deQLipVmDwaIIEWfyguLgmDr09fcz+zihk1RrWAIrQMlBYG0ysdksVBxgOXBa9w1lUOWeZll2tSHtIfgaC+6ivmzAAsjAKXbTbQOwR48QG6Xu3gR9xxWgXK9ldG19a+NLGlw6+dPGlhy8Nk16JpkFEDaJqEFmD6BpE2CDKBpE2iNYiWkuOR7RUO+9aRGsRrUW0FtFaRGsRbZNom0TblMwSbZNom0TbJNom0TaJtkm0NtHaRGsTrS0lJVqbaG2itYnWJlqbaFtE2yLaFtG2iLYl1US0LaJtEW2LaFtE2ybaNtG2ibZNtG2ibUsdE22baNtE2ybaDtF2iLZDtB2i7RBth2g70kBE2yHaDtF2ibZLtF2i7RJtl2i7RNsl2q60LtF2ibZHtD2i7RFtj2h7RNsj2h7R9oi2J6GhsCHBYUJSgdjeOw8OBzD3ehgk3n+KGGE4yb5jOzyqrAuul/Yczl1DgtXwxUgkLyzeqUELEW8o6Ceo1bDzappr/Fu7xdvdjX87Bf+GWqixWpCq/trfD60rAbXxjAncP7P8C8NW8OSjEcXHHQDUR6nhHh1+B/A+Ovw4XQOpvmO2HWcDqWeBVBrsBOGt4F9VZJS3PS5OsJ03Yi8cKdgJ/E3gGcHQe/KQwf9CbAIrZlZBxa4NOJR9pSm3vYHKAlTm8yXIoyFVfkulSbfvnMzg9XAstXKcNqG8NrM/tgYTTxwd/JwaxBTtFfjJgS8ZOA2wM67ufpcY/fTo8HNnJQg6tWaz7ZRtM4TfNiA4pRT7zSBOx+MwAnnIt7z9zq9WJdzstLIjbVyFlCh9ga5JDqnWIwB6v8dm1OH+GkDa3By0+AaQpwVIJxz1RUDi3KC9iGXFH+gZ4LMVal8lkzHaF8cUEYDmVBB5k/sDAwZ7sUDUVEADy4YUuUtHOdLlmGyebdS6pst4SVLV3LRH12zJjcMRP8FWXMv8B2/F3dI34Kq+pkcb74aCBbLI28HdmGsQ02uavGwvzQYxp4yYhc3bzw0NWc6VL7qvQoBVazWanbK9FM1NIfacEfALs3WuOeczLqVROOb1q6AwGPA5O4wMICdJfRAyXatr2oMNZE4PMi4T/uT/4yMfJbCRTOcdH+R8JV56NbttctYrw0vv5cWLacN/vRMvnRV3ZN3O3pavnGm/zi+dZT8dY6sGLZHlO7fkfu2jw8+yzZmqqle/YJ/nAbwCOj5MCSQfByvgYUMOYjUGfFCStdqbHOSYDwgAKAIe1eHalNcdn4nRmml9Aa8x8GnOJXvx5B2PtyXPPtusdbsdXtajs1/C53XWhwSQJImYk+SVp1y8fC/sLz4fCF+u3Xkrah5nPm7FBtX7Yugla+x/PbtO+XQYpGxqr7J5q+ZarNW2y2ze2th80eZsnDgeu6KewKjBe9/nwZA88LPbXk390InqwEy0zvC/pI4rOOmDB6lx7cKNrPOQMVfP2TKc/32Y+fYTw6NFW/PajlnSIGtt3Pox3XqfgVFq0qvHPEZXgSFfvsOIXx+zNOYlcT+/ZCHsy1+OEfWv460Ndf1JrW/VrHa/2bPKrL+pEU7L+hGP09FzMv8Nuvez2b+NjaV+v2GW2L+9mf3HfOQyCFLm16DaCqMkrmjb21yWQOKGBeIu94SDRVy1Mslb6euyeT4y+lMo6hx8me3fP+mDGO2zds3sOW1mlhl5szL7PIw8ZkNOyxT45qb4AD/AsMc3/jvTb1LDoeA/9qZf47ZrBtO6uBvWNA13+qdgWJc/zkMgSwr0PUQ6LNq1XqNtuY0yWLRf7nr/2aFRBz7wsdx1CIlpVexc5WY44tkK2bHRcYnGUGtT3JVP79MdATOH99VT2rhTfx/zxg8L231wteGL8Vzlr+OiU2s2zK7VLsPFS7xkuroHdFq4OCkGoAjIFxLw9CkRjc77/r8kUbrQMSCY1W9sXYNkgUW4ADEDiDw5Ym96z1GHwOiA6EGJ0Gi3SwHR2ziKUwPEzH6VcwPmx7y62ne8EQaXVMJItn37nV/Jh4Of2ZFoaKHIkjkLDSkg9gwbHUggO1a3yUrWpTqbhzxPjAlsGntg0TBadyLMjTQwLssrKdz/tzzGx9jjo6ohnwrP4v/JHvvs4KEdHafJm2UmbW0O9VllzlmDT9GvebbyinGZLqcJdo/OV5neE/p0S1Q9B6Z1BRsGYZwIJ9bN1amZHavTt8vM1dnMwPUn5rhiXTOODl7C6wpTDWLsBHP0R+Pqsz4k38VD1ZqdFussWq/7EjZgTjTZgDF3nZu8FLjjUASJgReLgMdxYXIVZl18dPBjYMTTr4Ihnt5UAf2CgBAWkQ/55CDUSpW3po8wn76PO6Qxdx7RKUmTWcGmJ9uYif/gYCPmZ4mAt85fPv8G1G8sW7l5FRMySuDxd2CGQvkZ/bA+lc7THjNa5kXyy1tb1w0H0z860ssBqBESx56sAORe3d3pV2GBoWCYUmtI7us+K4/ts842UTC8wtF3F1D7eaKWCh1MDv2QWkpyJ6ZWa6DkgVxqHmGtSiw6kLz4IcQcYIXaUJ8jP8fQzz/DkHSeGVw9ArJEXp4YO9Nv5BkH8O19B0e9nxre9I+Bp89AD0zoGbtC6ijC6QjVsbwD/i5ZZnHMIffRhEDmYODHtDoqz7XKFdQqFuWapODEIyD0STEw339gNM0/CTAfV8ds0eEajsfkSWwZe0PBwDhy5RWq/EdA6AtI5qpFw4MqEZb3ElIq+iKeoVo3fc4qHi57ORuDdgPXBaR3WB1qKPXktoBgiNZw8IQXr8Teaqf4ehjjNvFgWJ2HLJ0iA1NZLmHq7GZXFvF6DKh2Z1BFfvdH6uyxVwKYxSCEhCLOycTTByIvDC+fGtOvR/Tbg9ErGsQyFpLpI3z8YYZZoH8sSyPw+h4JLbGDmvm3m9feyECjTdk+VmSJAmgSTQ8c8EDxGBywXqLnMvVmMkmd4ZiIo/To4CHEEvxQqq+Etg6SayhAbyaWg7v7FTf4JAfq7KdEl+9Vj8WeCIb1IIxGzBcfUCg4o88oh44UmQER3QPiAe87nrmjRQVE0x9LlaAkb+qOR5tTA+Aku5OG2VthtANYc8IUsL8rBwPNyK8v0Lc+HzJnktFKWHs4l/+AugtDvzgF8TBeZ87Yy2ae1GduRpIY/MS9AAF9uMb6syFy0e2iS8k2ekTG3tHhI2Dzr9leDnf6FyNhfYTZ/sxBTf+EPb3DTwXZ/MvCtlI1X9HWP0sfpG6lvpHPE6IGZyLmOgFWPwzmZnJum5DO/0JFkLpmUSihE0UlE7mIc15TMXEN0hkoTmA8RPv9RFu0QBgf/DRW3nRRyEWJlKgx0joo18TYC9ETaTNbEBEYAgOFjLWLyiqecCgwSZCOKod3MGQT9R1Jm4uJHvffZ+h1fDYaw9XTryaG1as3zXqzoRr46QSuCijhQEXivnd/UpCzxCAzZCzjHVkMPNnQk/deYj/NSLlcuRgdfECIfO5wxio9OSidktoPV1eal79IF0CMzTT+PmTGSt0qS6JTrO+T93oondx4URoXHRRhs4qHkeLKNh5tCpojP5Ivfwwgx4MoscuNLDuuztwjTBaZe2O0KQvzC3JjRLkoYtb3Odw6SSOOUS2m+dGns+4kHAO+lxi0eE9l9H3Zhw8K5iOZ3OmPYi65VDrDseclPoapgIsf4AI950O/QygNlBw2HmyRO1NUmjrOWfb25P4B4H7I607o8rrLEyZ8XTFoPy1cgG8c4gmzmncsSS5V/M8yBCDvR+Et0PkyD7IuclDzSUsDJPt6BrIHUk+MiOWCW1gf6E9Kj4hGsZa704RWRZ7czVw55SQOHWnoo4/W7Tia/pmk/ZR6JnJmFUVFeH2mxPsy06+SXaYekMgVFmzwxMR9deiyUodu2L7PnJ1aP9wrt66t5z3IUP4AH2FuwTTE4CeOwu7Fa6+rCTHLZAqRcNGAUPIm4Ug+5aJhAADzIEv7chvPvFZ+Iux8spoL0tZCvqTGIgFzHTQa7nXBpsfSzIwqN5mQIMiLBcYy0MmCpBi7EXMqWcwrebqdh0U73gAy2pzrTjGUYc7RD8MdQ7Zxi6kzaj8d+yHDpRlSsKP2XGqOYvoIJJCeajc7XRMdpouO9+NEN4jMtjNMLQ1UMqRSi0LlqeVFYi4TOr7rtLyoqqM3rm1fPL91Xm9eSN7UJBQjHqZJfevqzbpt2ksnjLx6lPk/rXag/IEmQxaNZ6onKeemzBjn8wjxqUypsi5ODZbPx+VTpVeMxzvkzt5PUVNQ7jwSck7UVTIxQnQFpC81CMaURCSTetGHLxM3YpDP5C2WgsC49vodm/MgVVlSyKBaqIlym+liLXOM5L7kYEryFqXTN3gSTeTI8ppMHMKlT90pqRKWJHw0xnQedf5F0QNS3g/kddxUpstEaahKtfCOiYyFffIz+q0eK3vr86m6tKlRrggtMKwLPrkS7KL5M1DrdSB6KSbvsUsLHREpTQK3TAtSaj1pzSatjpBsqEXMF3VQIoo23WdSwXzPpcJc+u0slKlLXBED7gLuJDIIDBGKdZ8rhkvROpIpNwEgoIhYnKgyky44+ZNEMdW7UwhGEcHD5kJQpgx2EFIFMBpL0S1TUiX/XsHht8bN/7haYD+7QOcQAtQuaKBYwxStsS4sFD2k7NQwyn0J231VLtBB+XkkaFEkyPsrSCU1qrQoffXJPaM6Z1tveZR2U4pMJyrpmYHLcGkC5g4Tv36U896l852z3hpOuQ/V8e/Gq09++/YZlWQnkaDkf8djIv/bANXSHlth7KKbmKlajd+WKao2N6WJ3JS0nmee9KgtHsXjG68mAoMucVo14nQ0YtGkmp9S4UpN0iEFoNsvgjMF1Y9ZFHN5O0iGYd7TZpoVgC5v7MjZQNkPNbNkNQjl3Uwu7Axfffp9XuPGOFNlXKM0XPYroJBzdkAIpRx8vSvyZ4Yh2ca7qwoYL396j8D4cxmU0QrUzCF975f3mrBuirCjXayGytzrk7vhlGIOBWeQYiacdZy2t9VS25GWNnjJheo7Exddo5z/WRBZHiwKfUKss+emhdanKG8/5sJZWudbqOIckfLK3/7rf14B7Ydz4khT7c41ewLjjTevXs2yPbOYWhfu++aVVb1ezTPlNiQkUkq8vr8235jPxWzqTuuCj2cQ7WHvbO4BoGT6xxG+P/h5RDIkT79/Sq4Ki4ZlrCMS85Z0Sc+91BNgOLusKyZDAPb4rzKwWUonz7p1Oh0gNm6JBOY7S9hc9FzTY1255ECIlNNu6byaTSHsSrJELSD5VPXpsyoXDZ3sZcpOtQ01Kl+AwR+A/7oUO2zMq3BLJ42Xrwos/JUWiqZgiDUBDSKp4qZDAC8oGoQ+UA5BO+iH2v3Sjyo9HR3+DtWBKeA4Ch0OQrr13Ar1IJT/x79exN2FpAlyh0VVq/xJyUoK0U1D1yhkL/UBS3PFXOLmXPqv9bG9LDJ9jkH427nFOvIa+s4KNMyudA6zsjkL0lBK3J1bsdCa6hd/qRI43VdgObMP8T90ds6sXOUp6zIXc6kOpbmXINl0qfEPEwBP5/WiMB16YyjS6C8FcYP7bBzP2Wc2llpdU+FQJT662eYaVtXsORTUhjTRl9KFQ71IDzngzgffP1lPKxepPV+Qyq6venamT/No7LMgwL6UXpne4v1YJLygCzUA/a0r5ES5MvlpWYKWUNKHruVunq7p+tAbmKqOUzFV5QolKwXkwBd8cvcs5gyXCeUUNA++DQpLNPJvbqi+HXegQomrgMChXKrPSq9s+Qd3av1B5H/fiZw33kxBc5d0RxOvOofG3PNg/j1bH53zKTnXtnzoAOYHl5ULOIf3qAKhnowynMx2snZ3xAYD4RBTWmtY44n6dqjVBwozD2TLZEWM0aMKcTnrn2HIF3nG3qVY89r0MWAO3Q85WOWUlZ8VI2yL5gfJqsavjh6Xj/1wskKC+oUrtQsXn023WdFUny2P3alWbjGYv5E8C+z/AHoy450=</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -1654,7 +1654,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -1701,7 +1701,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -1748,7 +1748,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K23" s="3" t="inlineStr">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K24" s="3" t="inlineStr">
@@ -2030,7 +2030,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K25" s="3" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K26" s="3" t="inlineStr">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K27" s="3" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K29" s="3" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K30" s="3" t="inlineStr">
@@ -2312,7 +2312,7 @@
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K31" s="3" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K32" s="3" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K33" s="3" t="inlineStr">
@@ -2453,7 +2453,7 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K34" s="3" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K35" s="3" t="inlineStr">
@@ -2547,7 +2547,7 @@
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K36" s="3" t="inlineStr">
@@ -2594,7 +2594,7 @@
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K37" s="3" t="inlineStr">
@@ -2641,7 +2641,7 @@
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K38" s="3" t="inlineStr">
@@ -2688,7 +2688,7 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K39" s="3" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>draft</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="K40" s="3" t="inlineStr">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-1</t>
+          <t>approved 1, draft 0, rejected 0; story US-1</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 2, rejected 0; story US-1</t>
+          <t>approved 2, draft 0, rejected 0; story US-1</t>
         </is>
       </c>
     </row>
@@ -6352,7 +6352,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-1</t>
+          <t>approved 1, draft 0, rejected 0; story US-1</t>
         </is>
       </c>
     </row>
@@ -6374,7 +6374,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-1</t>
+          <t>approved 1, draft 0, rejected 0; story US-1</t>
         </is>
       </c>
     </row>
@@ -6396,7 +6396,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 2, rejected 0; story US-1</t>
+          <t>approved 2, draft 0, rejected 0; story US-1</t>
         </is>
       </c>
     </row>
@@ -6418,7 +6418,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-1</t>
+          <t>approved 1, draft 0, rejected 0; story US-1</t>
         </is>
       </c>
     </row>
@@ -6462,7 +6462,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-1</t>
+          <t>approved 1, draft 0, rejected 0; story US-1</t>
         </is>
       </c>
     </row>
@@ -6484,7 +6484,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 2, rejected 0; story US-1</t>
+          <t>approved 2, draft 0, rejected 0; story US-1</t>
         </is>
       </c>
     </row>
@@ -6506,7 +6506,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 4, rejected 0; story US-2</t>
+          <t>approved 4, draft 0, rejected 0; story US-2</t>
         </is>
       </c>
     </row>
@@ -6528,7 +6528,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 3, rejected 0; story US-2</t>
+          <t>approved 3, draft 0, rejected 0; story US-2</t>
         </is>
       </c>
     </row>
@@ -6572,7 +6572,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-2</t>
+          <t>approved 1, draft 0, rejected 0; story US-2</t>
         </is>
       </c>
     </row>
@@ -6638,7 +6638,7 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 2, rejected 0; story US-2</t>
+          <t>approved 2, draft 0, rejected 0; story US-2</t>
         </is>
       </c>
     </row>
@@ -6704,7 +6704,7 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-2</t>
+          <t>approved 1, draft 0, rejected 0; story US-2</t>
         </is>
       </c>
     </row>
@@ -6748,7 +6748,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 2, rejected 0; story US-3</t>
+          <t>approved 2, draft 0, rejected 0; story US-3</t>
         </is>
       </c>
     </row>
@@ -6770,7 +6770,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 2, rejected 0; story US-3</t>
+          <t>approved 2, draft 0, rejected 0; story US-3</t>
         </is>
       </c>
     </row>
@@ -6924,7 +6924,7 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-3</t>
+          <t>approved 1, draft 0, rejected 0; story US-3</t>
         </is>
       </c>
     </row>
@@ -6946,7 +6946,7 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-4</t>
+          <t>approved 1, draft 0, rejected 0; story US-4</t>
         </is>
       </c>
     </row>
@@ -6990,7 +6990,7 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-4</t>
+          <t>approved 1, draft 0, rejected 0; story US-4</t>
         </is>
       </c>
     </row>
@@ -7034,7 +7034,7 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-4</t>
+          <t>approved 1, draft 0, rejected 0; story US-4</t>
         </is>
       </c>
     </row>
@@ -7166,7 +7166,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-5</t>
+          <t>approved 1, draft 0, rejected 0; story US-5</t>
         </is>
       </c>
     </row>
@@ -7188,7 +7188,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-5</t>
+          <t>approved 1, draft 0, rejected 0; story US-5</t>
         </is>
       </c>
     </row>
@@ -7342,7 +7342,7 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-6</t>
+          <t>approved 1, draft 0, rejected 0; story US-6</t>
         </is>
       </c>
     </row>
@@ -7408,7 +7408,7 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-6</t>
+          <t>approved 1, draft 0, rejected 0; story US-6</t>
         </is>
       </c>
     </row>
@@ -7452,7 +7452,7 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-6</t>
+          <t>approved 1, draft 0, rejected 0; story US-6</t>
         </is>
       </c>
     </row>
@@ -7474,7 +7474,7 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-6</t>
+          <t>approved 1, draft 0, rejected 0; story US-6</t>
         </is>
       </c>
     </row>
@@ -7518,7 +7518,7 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-6</t>
+          <t>approved 1, draft 0, rejected 0; story US-6</t>
         </is>
       </c>
     </row>
@@ -7606,7 +7606,7 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-7</t>
+          <t>approved 1, draft 0, rejected 0; story US-7</t>
         </is>
       </c>
     </row>
@@ -7694,7 +7694,7 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-7</t>
+          <t>approved 1, draft 0, rejected 0; story US-7</t>
         </is>
       </c>
     </row>
@@ -7738,7 +7738,7 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-7</t>
+          <t>approved 1, draft 0, rejected 0; story US-7</t>
         </is>
       </c>
     </row>
@@ -7782,7 +7782,7 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>approved 0, draft 1, rejected 0; story US-8</t>
+          <t>approved 1, draft 0, rejected 0; story US-8</t>
         </is>
       </c>
     </row>

</xml_diff>